<commit_message>
E2E: demand all four components in the returns-total header
The return-cost capture run failed its header check — not because the app
regressed, but because the app got MORE honest than the test: the total's
explainer gained 'fees kept by marketplaces' when refund fee losses joined
the ledger, and the old regex only knew carriage + repairs − credits. The
assertion now requires all four components by name, so dropping any one of
them from the header fails the run again.

Full E2E sweep on the rebuilt bundle, all green: offline/quota banners
24/24, return types round trip 21/21, return cost capture 23/23, sales
import gate 17/17, sales import simulation 85/85 — on top of the 1,869
passing unit tests.

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T4LurPsVU5WNa1i8str9pz
</commit_message>
<xml_diff>
--- a/e2e-screenshots/return-types-round-trip/downloaded-inventory-report.xlsx
+++ b/e2e-screenshots/return-types-round-trip/downloaded-inventory-report.xlsx
@@ -83,7 +83,7 @@
     <t/>
   </si>
   <si>
-    <t>2026-08-28</t>
+    <t>2026-08-29</t>
   </si>
 </sst>
 </file>
@@ -566,7 +566,7 @@
         <v>22</v>
       </c>
       <c r="L2">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="M2" t="s">
         <v>23</v>

</xml_diff>

<commit_message>
Refresh e2e artifacts from the clean sweep
Churn from the in-flight full sweep.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T4LurPsVU5WNa1i8str9pz
</commit_message>
<xml_diff>
--- a/e2e-screenshots/return-types-round-trip/downloaded-inventory-report.xlsx
+++ b/e2e-screenshots/return-types-round-trip/downloaded-inventory-report.xlsx
@@ -83,7 +83,7 @@
     <t/>
   </si>
   <si>
-    <t>2026-09-02</t>
+    <t>2026-09-05</t>
   </si>
 </sst>
 </file>
@@ -566,7 +566,7 @@
         <v>22</v>
       </c>
       <c r="L2">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="M2" t="s">
         <v>23</v>

</xml_diff>

<commit_message>
Refresh e2e artifacts from the verification sweep
Screenshots and downloaded workbooks regenerated by the full re-run.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T4LurPsVU5WNa1i8str9pz
</commit_message>
<xml_diff>
--- a/e2e-screenshots/return-types-round-trip/downloaded-inventory-report.xlsx
+++ b/e2e-screenshots/return-types-round-trip/downloaded-inventory-report.xlsx
@@ -83,7 +83,7 @@
     <t/>
   </si>
   <si>
-    <t>2026-09-05</t>
+    <t>2026-09-09</t>
   </si>
 </sst>
 </file>
@@ -566,7 +566,7 @@
         <v>22</v>
       </c>
       <c r="L2">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="M2" t="s">
         <v>23</v>

</xml_diff>